<commit_message>
Split Design Task Hub into three interfaces with an approval funnel
Task Creation (#pm), Designer Tracker (#designer) and Owner Dashboard (#owner)
are now separate interfaces with their own links, headers and navigation.
PMs build requests with dependent 4E line and product dropdowns and detailed
subtasks, each with its own designer and timeline; requests wait in the
owner's task funnel (approve, request changes, reject) and only approved
subtasks become Tracker tasks. Designer progress and leave move to per-person
paths so database rules keep each group to its own writes. The workbook gains
a Task Funnel sheet, 4E and request columns on Task Details, and funnel and
4E tables on the Dashboard.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RGr5xFPprK8caaFpz2CWq4
</commit_message>
<xml_diff>
--- a/designer-task-hub/workbook/template.xlsx
+++ b/designer-task-hub/workbook/template.xlsx
@@ -20,6 +20,7 @@
     <sheet name="Dashboard" sheetId="7" r:id="rId21"/>
     <sheet name="Task Details" sheetId="8" r:id="rId22"/>
     <sheet name="Daily Log" sheetId="9" r:id="rId23"/>
+    <sheet name="Task Funnel" sheetId="10" r:id="rId24"/>
   </sheets>
   <calcPr calcId="181029" fullCalcOnLoad="1"/>
   <extLst>
@@ -19733,7 +19734,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P145"/>
+  <dimension ref="A1:P160"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -21429,6 +21430,199 @@
       </c>
       <c r="G145" s="60">
         <f>IF($A145="","",SUMIFS(tblTasks[Estimated Effort (Hrs)],tblTasks[Project],$A145))</f>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Request Funnel</t>
+        </is>
+      </c>
+      <c r="B148" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subtasks</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Awaiting approval</t>
+        </is>
+      </c>
+      <c r="B149" s="12">
+        <f>COUNTIFS('Task Funnel'!$O:$O,$A149)</f>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Changes requested</t>
+        </is>
+      </c>
+      <c r="B150" s="12">
+        <f>COUNTIFS('Task Funnel'!$O:$O,$A150)</f>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="B151" s="12">
+        <f>COUNTIFS('Task Funnel'!$O:$O,$A151)</f>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+      <c r="B152" s="12">
+        <f>COUNTIFS('Task Funnel'!$O:$O,$A152)</f>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4E Line</t>
+        </is>
+      </c>
+      <c r="B154" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tasks</t>
+        </is>
+      </c>
+      <c r="C154" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="D154" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Est. Hours</t>
+        </is>
+      </c>
+      <c r="E154" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hours Logged</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evaluate</t>
+        </is>
+      </c>
+      <c r="B155" s="12">
+        <f>COUNTIFS('Task Details'!$Q:$Q,$A155)</f>
+      </c>
+      <c r="C155" s="12">
+        <f>B155-COUNTIFS('Task Details'!$Q:$Q,$A155,'Task Details'!$H:$H,"Done*")</f>
+      </c>
+      <c r="D155" s="60">
+        <f>SUMIFS('Task Details'!$I:$I,'Task Details'!$Q:$Q,$A155)</f>
+      </c>
+      <c r="E155" s="60">
+        <f>SUMIFS('Task Details'!$K:$K,'Task Details'!$Q:$Q,$A155)</f>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Educate</t>
+        </is>
+      </c>
+      <c r="B156" s="12">
+        <f>COUNTIFS('Task Details'!$Q:$Q,$A156)</f>
+      </c>
+      <c r="C156" s="12">
+        <f>B156-COUNTIFS('Task Details'!$Q:$Q,$A156,'Task Details'!$H:$H,"Done*")</f>
+      </c>
+      <c r="D156" s="60">
+        <f>SUMIFS('Task Details'!$I:$I,'Task Details'!$Q:$Q,$A156)</f>
+      </c>
+      <c r="E156" s="60">
+        <f>SUMIFS('Task Details'!$K:$K,'Task Details'!$Q:$Q,$A156)</f>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Experience</t>
+        </is>
+      </c>
+      <c r="B157" s="12">
+        <f>COUNTIFS('Task Details'!$Q:$Q,$A157)</f>
+      </c>
+      <c r="C157" s="12">
+        <f>B157-COUNTIFS('Task Details'!$Q:$Q,$A157,'Task Details'!$H:$H,"Done*")</f>
+      </c>
+      <c r="D157" s="60">
+        <f>SUMIFS('Task Details'!$I:$I,'Task Details'!$Q:$Q,$A157)</f>
+      </c>
+      <c r="E157" s="60">
+        <f>SUMIFS('Task Details'!$K:$K,'Task Details'!$Q:$Q,$A157)</f>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enable</t>
+        </is>
+      </c>
+      <c r="B158" s="12">
+        <f>COUNTIFS('Task Details'!$Q:$Q,$A158)</f>
+      </c>
+      <c r="C158" s="12">
+        <f>B158-COUNTIFS('Task Details'!$Q:$Q,$A158,'Task Details'!$H:$H,"Done*")</f>
+      </c>
+      <c r="D158" s="60">
+        <f>SUMIFS('Task Details'!$I:$I,'Task Details'!$Q:$Q,$A158)</f>
+      </c>
+      <c r="E158" s="60">
+        <f>SUMIFS('Task Details'!$K:$K,'Task Details'!$Q:$Q,$A158)</f>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GENIE Platform</t>
+        </is>
+      </c>
+      <c r="B159" s="12">
+        <f>COUNTIFS('Task Details'!$Q:$Q,$A159)</f>
+      </c>
+      <c r="C159" s="12">
+        <f>B159-COUNTIFS('Task Details'!$Q:$Q,$A159,'Task Details'!$H:$H,"Done*")</f>
+      </c>
+      <c r="D159" s="60">
+        <f>SUMIFS('Task Details'!$I:$I,'Task Details'!$Q:$Q,$A159)</f>
+      </c>
+      <c r="E159" s="60">
+        <f>SUMIFS('Task Details'!$K:$K,'Task Details'!$Q:$Q,$A159)</f>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Other</t>
+        </is>
+      </c>
+      <c r="B160" s="12">
+        <f>COUNTIFS('Task Details'!$Q:$Q,$A160)</f>
+      </c>
+      <c r="C160" s="12">
+        <f>B160-COUNTIFS('Task Details'!$Q:$Q,$A160,'Task Details'!$H:$H,"Done*")</f>
+      </c>
+      <c r="D160" s="60">
+        <f>SUMIFS('Task Details'!$I:$I,'Task Details'!$Q:$Q,$A160)</f>
+      </c>
+      <c r="E160" s="60">
+        <f>SUMIFS('Task Details'!$K:$K,'Task Details'!$Q:$Q,$A160)</f>
       </c>
     </row>
   </sheetData>
@@ -21458,7 +21652,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:T4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -21477,6 +21671,10 @@
     <col min="14" max="14" width="14" customWidth="1"/>
     <col min="15" max="15" width="13" customWidth="1"/>
     <col min="16" max="16" width="36" customWidth="1"/>
+    <col min="17" max="17" width="12" customWidth="1"/>
+    <col min="18" max="18" width="30" customWidth="1"/>
+    <col min="19" max="19" width="11" customWidth="1"/>
+    <col min="20" max="20" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -21574,9 +21772,29 @@
           <t xml:space="preserve">Brief / Link</t>
         </is>
       </c>
+      <c r="Q4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4E Line</t>
+        </is>
+      </c>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Master Task Title</t>
+        </is>
+      </c>
+      <c r="S4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Request ID</t>
+        </is>
+      </c>
+      <c r="T4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Approved On</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:P4"/>
+  <autoFilter ref="A4:T4"/>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -21668,4 +21886,141 @@
   <autoFilter ref="A4:J4"/>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:R4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="1" max="1" width="11" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="30" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="40" customWidth="1"/>
+    <col min="11" max="11" width="13" customWidth="1"/>
+    <col min="12" max="12" width="12" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="14" max="14" width="10" customWidth="1"/>
+    <col min="15" max="15" width="17" customWidth="1"/>
+    <col min="16" max="16" width="12" customWidth="1"/>
+    <col min="17" max="17" width="36" customWidth="1"/>
+    <col min="18" max="18" width="9" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Task Funnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Every request PMs submitted, one row per subtask, with your decision. Approved subtasks become Tracker rows (Task ID).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Request ID</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Submitted</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PM</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4E Line</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Project</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Master Task</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Priority</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subtask</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detail</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Designer</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Start</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">End</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Est. Hours</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Status</t>
+        </is>
+      </c>
+      <c r="P4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decided On</t>
+        </is>
+      </c>
+      <c r="Q4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Owner Note</t>
+        </is>
+      </c>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Task ID</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:R4"/>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>